<commit_message>
#3 PCB updated with toggle switch Deliverables generated
</commit_message>
<xml_diff>
--- a/Design-Files/PowerCutMonitor-v1.0 (Contactless Version)/Deliverables/BOM/Client_BOM.xlsx
+++ b/Design-Files/PowerCutMonitor-v1.0 (Contactless Version)/Deliverables/BOM/Client_BOM.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="149">
   <si>
     <t>#</t>
   </si>
@@ -396,6 +396,18 @@
   </si>
   <si>
     <t>Omron</t>
+  </si>
+  <si>
+    <t>SW3</t>
+  </si>
+  <si>
+    <t>3A Direct Insert Single Pole Double Throw (SPDT) 125V Black 10,000 times Plugin Slide Switches ROHS</t>
+  </si>
+  <si>
+    <t>SS-12D10L9</t>
+  </si>
+  <si>
+    <t>XKB Connectivity</t>
   </si>
   <si>
     <t>Module</t>
@@ -1205,7 +1217,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1240,6 +1252,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1570,7 +1591,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -1594,11 +1615,11 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+    </row>
+    <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1631,7 +1652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" ht="15.75" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
         <f>ROW(B3)-ROW($B$2)</f>
@@ -1759,7 +1780,7 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" ht="15.75" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f>ROW(B7)-ROW($B$2)</f>
@@ -1887,7 +1908,7 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" ht="15.75" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
         <f>ROW(B11)-ROW($B$2)</f>
@@ -1919,7 +1940,7 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" ht="15.75" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
         <f>ROW(B12)-ROW($B$2)</f>
@@ -2047,7 +2068,7 @@
       </c>
       <c r="K15" s="9"/>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" ht="15.75" spans="1:11">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
         <f>ROW(B16)-ROW($B$2)</f>
@@ -2335,37 +2356,34 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" ht="36.75" spans="1:11">
       <c r="A25" s="2"/>
-      <c r="B25" s="7">
-        <f>ROW(B25)-ROW($B$2)</f>
-        <v>23</v>
-      </c>
-      <c r="C25" s="8" t="s">
+      <c r="B25" s="7"/>
+      <c r="C25" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="16" t="s">
         <v>124</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="F25" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="H25" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="H25" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="I25" s="10" t="s">
+      <c r="I25" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="15">
         <v>1</v>
       </c>
-      <c r="K25" s="9"/>
+      <c r="K25" s="15"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2"/>
@@ -2373,95 +2391,127 @@
         <f>ROW(B26)-ROW($B$2)</f>
         <v>24</v>
       </c>
-      <c r="C26" s="11" t="s">
+      <c r="C26" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="E26" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="F26" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="H26" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="G26" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="I26" s="13" t="s">
+      <c r="I26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="12"/>
-    </row>
-    <row r="27" spans="1:11">
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27" ht="15.75" spans="1:11">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
         <f>ROW(B27)-ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="F27" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="G27" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="H27" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="G27" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="I27" s="10" t="s">
+      <c r="I27" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J27" s="9">
+      <c r="J27" s="12">
         <v>1</v>
       </c>
-      <c r="K27" s="9"/>
-    </row>
-    <row r="28" ht="36.75" spans="1:11">
+      <c r="K27" s="12"/>
+    </row>
+    <row r="28" ht="15.75" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
         <f>ROW(B28)-ROW($B$2)</f>
         <v>26</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="F28" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="G28" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="F28" s="12" t="s">
+      <c r="H28" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J28" s="9">
+        <v>1</v>
+      </c>
+      <c r="K28" s="9"/>
+    </row>
+    <row r="29" ht="36.75" spans="1:11">
+      <c r="A29" s="2"/>
+      <c r="B29" s="7">
+        <f>ROW(B29)-ROW($B$2)</f>
+        <v>27</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="F29" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="G28" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="H28" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="I28" s="13" t="s">
+      <c r="G29" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="I29" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J28" s="12">
+      <c r="J29" s="12">
         <v>1</v>
       </c>
-      <c r="K28" s="12"/>
+      <c r="K29" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>